<commit_message>
Docs : ajout des sprints individuel
</commit_message>
<xml_diff>
--- a/docs/DiagrammeGantt.xlsx
+++ b/docs/DiagrammeGantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabinb/IUT/S5/SAE/Application IA/11_Doc2Quiz/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C1FD38-BE1C-C04C-9004-760A9639DD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD5D996-8D43-C749-AF5C-A0F3BD356FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17460" xr2:uid="{33E6F111-0219-404F-8A7B-D068A4E95F65}"/>
   </bookViews>
@@ -3229,7 +3229,7 @@
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="9"/>
@@ -4879,7 +4879,7 @@
       <c r="C30" s="30"/>
       <c r="D30" s="30"/>
       <c r="E30" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="31"/>

</xml_diff>